<commit_message>
fix(data): stop the example workbook failing its own import
make-example.mjs wrote "Por confirmar" as a placeholder Profesor name for a
session with no teacher, but buildSchedule reads any non-empty cell there as
a teacher name and rejects one that names nobody. Writing nothing instead
matches how a real workbook represents an unassigned session.
</commit_message>
<xml_diff>
--- a/content/ejemplo-completo.xlsx
+++ b/content/ejemplo-completo.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="141">
   <si>
     <t>Dia</t>
   </si>
@@ -101,7 +101,7 @@
     <t>Sexy Style</t>
   </si>
   <si>
-    <t>Por confirmar</t>
+    <t/>
   </si>
   <si>
     <t>21:00</t>
@@ -270,9 +270,6 @@
   </si>
   <si>
     <t>Izquierdo</t>
-  </si>
-  <si>
-    <t/>
   </si>
   <si>
     <t>Ejemplo: dos o tres líneas contando su trayectoria. Reemplaza este texto.</t>
@@ -1890,249 +1887,249 @@
         <v>30</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F2" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="G2" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="H2" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J2" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="3" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C3" s="2" t="s">
         <v>63</v>
       </c>
       <c r="D3" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F3" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E3" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H3" s="2" t="s">
+      <c r="I3" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I3" s="2" t="s">
+      <c r="J3" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="4" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>59</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F4" s="2" t="s">
+      <c r="G4" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="H4" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="I4" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="J4" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="5" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C5" s="2" t="s">
         <v>65</v>
       </c>
       <c r="D5" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F5" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E5" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F5" s="2" t="s">
+      <c r="G5" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="2" t="s">
+      <c r="H5" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H5" s="2" t="s">
+      <c r="I5" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I5" s="2" t="s">
+      <c r="J5" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="6" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="G6" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="H6" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="I6" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="J6" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="7" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>53</v>
       </c>
       <c r="D7" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E7" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F7" s="2" t="s">
+      <c r="G7" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G7" s="2" t="s">
+      <c r="H7" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I7" s="2" t="s">
+      <c r="J7" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="8" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>57</v>
       </c>
       <c r="D8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F8" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E8" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F8" s="2" t="s">
+      <c r="G8" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="H8" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="I8" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I8" s="2" t="s">
+      <c r="J8" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="9" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C9" s="2" t="s">
         <v>55</v>
       </c>
       <c r="D9" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E9" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F9" s="2" t="s">
+      <c r="G9" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="I9" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I9" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="10" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2140,31 +2137,31 @@
         <v>31</v>
       </c>
       <c r="B10" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="D10" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="D10" s="2" t="s">
-        <v>100</v>
-      </c>
       <c r="E10" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F10" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="G10" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="H10" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="I10" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="J10" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="11" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2172,31 +2169,31 @@
         <v>12</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C11" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E11" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F11" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F11" s="2" t="s">
+      <c r="G11" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G11" s="2" t="s">
+      <c r="H11" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H11" s="2" t="s">
+      <c r="I11" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I11" s="2" t="s">
+      <c r="J11" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="12" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2204,31 +2201,31 @@
         <v>18</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C12" s="2" t="s">
         <v>17</v>
       </c>
       <c r="D12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F12" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F12" s="2" t="s">
+      <c r="G12" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="H12" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H12" s="2" t="s">
+      <c r="I12" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I12" s="2" t="s">
+      <c r="J12" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="13" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2236,31 +2233,31 @@
         <v>23</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C13" s="2" t="s">
         <v>22</v>
       </c>
       <c r="D13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F13" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E13" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F13" s="2" t="s">
+      <c r="G13" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G13" s="2" t="s">
+      <c r="H13" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H13" s="2" t="s">
+      <c r="I13" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I13" s="2" t="s">
+      <c r="J13" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="14" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2268,31 +2265,31 @@
         <v>32</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C14" s="2" t="s">
         <v>30</v>
       </c>
       <c r="D14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F14" s="2" t="s">
+      <c r="G14" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G14" s="2" t="s">
+      <c r="H14" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H14" s="2" t="s">
+      <c r="I14" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I14" s="2" t="s">
+      <c r="J14" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="15" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2300,31 +2297,31 @@
         <v>39</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>38</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E15" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F15" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="F15" s="2" t="s">
+      <c r="G15" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G15" s="2" t="s">
+      <c r="H15" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I15" s="2" t="s">
+      <c r="J15" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="16" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2332,31 +2329,31 @@
         <v>45</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>44</v>
       </c>
       <c r="D16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="F16" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E16" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" s="2" t="s">
+      <c r="G16" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G16" s="2" t="s">
+      <c r="H16" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H16" s="2" t="s">
+      <c r="I16" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I16" s="2" t="s">
+      <c r="J16" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
     <row r="17" ht="64" customHeight="1" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -2364,31 +2361,31 @@
         <v>36</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C17" s="2" t="s">
         <v>35</v>
       </c>
       <c r="D17" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F17" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E17" s="2" t="s">
-        <v>85</v>
-      </c>
-      <c r="F17" s="2" t="s">
+      <c r="G17" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="G17" s="2" t="s">
+      <c r="H17" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="H17" s="2" t="s">
+      <c r="I17" s="2" t="s">
         <v>88</v>
       </c>
-      <c r="I17" s="2" t="s">
+      <c r="J17" s="2" t="s">
         <v>89</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>90</v>
       </c>
     </row>
   </sheetData>
@@ -2411,58 +2408,58 @@
   <sheetData>
     <row r="1" spans="1:4" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>109</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="D1" s="1" t="s">
         <v>111</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B2" t="s">
         <v>113</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>114</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>115</v>
-      </c>
-      <c r="D2" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>116</v>
+      </c>
+      <c r="B3" t="s">
         <v>117</v>
-      </c>
-      <c r="B3" t="s">
-        <v>118</v>
       </c>
       <c r="C3" t="s">
         <v>80</v>
       </c>
       <c r="D3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>119</v>
+      </c>
+      <c r="B4" t="s">
         <v>120</v>
-      </c>
-      <c r="B4" t="s">
-        <v>121</v>
       </c>
       <c r="C4" t="s">
         <v>81</v>
       </c>
       <c r="D4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -2482,10 +2479,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2493,55 +2490,55 @@
         <v>47</v>
       </c>
       <c r="B2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>125</v>
+      </c>
+      <c r="B3" t="s">
         <v>126</v>
-      </c>
-      <c r="B3" t="s">
-        <v>127</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B4" t="s">
         <v>128</v>
-      </c>
-      <c r="B4" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>129</v>
+      </c>
+      <c r="B5" t="s">
         <v>130</v>
-      </c>
-      <c r="B5" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>131</v>
+      </c>
+      <c r="B6" t="s">
         <v>132</v>
-      </c>
-      <c r="B6" t="s">
-        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" t="s">
         <v>134</v>
-      </c>
-      <c r="B7" t="s">
-        <v>135</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" t="s">
         <v>136</v>
-      </c>
-      <c r="B8" t="s">
-        <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -2549,7 +2546,7 @@
         <v>80</v>
       </c>
       <c r="B9" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -2557,23 +2554,23 @@
         <v>81</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>137</v>
+      </c>
+      <c r="B11" t="s">
         <v>138</v>
-      </c>
-      <c r="B11" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>139</v>
+      </c>
+      <c r="B12" t="s">
         <v>140</v>
-      </c>
-      <c r="B12" t="s">
-        <v>141</v>
       </c>
     </row>
   </sheetData>

</xml_diff>